<commit_message>
Atualizar restos.xlsx - 23/06/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -55384,13 +55384,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{848A4E03-A3A4-456B-833F-B6CE9B5C20F4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B83B2EB7-5FA5-4401-9F2B-91AB4200891B}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54D9BA03-E1B7-45F4-AF92-B16A677BB360}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FBA08EF-CA25-4038-89B5-E8A25E90F42E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC28E1BB-02E4-4BCB-838E-D15CC12E2742}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DC5007B0-140E-48DC-9E44-1B35A746815D}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 24/06/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -55384,13 +55384,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B83B2EB7-5FA5-4401-9F2B-91AB4200891B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8DBB914C-A893-45C7-A4A2-2BFCB877BE61}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FBA08EF-CA25-4038-89B5-E8A25E90F42E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C860D57-5782-4EBC-97DF-DAE8062A870C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DC5007B0-140E-48DC-9E44-1B35A746815D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{89B69F17-26E9-45F0-935E-C9C87671F36F}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 01/07/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -56831,13 +56831,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C804802F-62BC-4BB2-98EB-78CC7C7CDE02}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{134E88CE-42BF-4479-838D-7F59E74377A1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F10094E-DF75-461F-829D-8E1B44897AE5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12E6F0C3-2C4C-4551-9064-0CEA765390D8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBA07D4E-45A1-4EAA-8CDF-36F0D325D8D0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACE376E2-6650-4666-8D26-DF70AA7788E9}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 02/07/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -56831,13 +56831,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{134E88CE-42BF-4479-838D-7F59E74377A1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECE0F1CF-0C7D-4751-B053-088A3BF4E4C2}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12E6F0C3-2C4C-4551-9064-0CEA765390D8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3078EF0A-A0C3-458F-89A5-712A566DBA6C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACE376E2-6650-4666-8D26-DF70AA7788E9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6BF5E4C6-9022-4C54-BDB6-5278164D2B97}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 09/07/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -55384,13 +55384,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0EAC3EC0-B65B-4E43-9C08-63037E8B50F9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBE7AA0B-0FA2-4C70-8B97-18443C35D8A7}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70B70EF7-285E-41AE-93AB-C5B4EF3C47D6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF23F52C-8121-4857-A8C3-50B639470488}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D28BEFBB-72B9-4FCE-8444-9EA010C76C6F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{530591B9-C9B5-48EC-BDD0-954252D15EA4}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 16/07/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -56831,13 +56831,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{10FAC376-7E52-4CB8-A144-CB9371FCB60A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6155A34-3B57-4253-A425-7BD676AE59B7}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E855ACE5-C059-4788-8C1D-34B6E37654F5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5380A27B-2D7E-4002-B459-EBE5044FFD9F}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{997F833B-4DC6-467B-AD6C-88FF8D15237A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D9CF7E2-B40D-410E-9074-10945FA93BCC}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 17/07/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -56831,13 +56831,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6155A34-3B57-4253-A425-7BD676AE59B7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DAFC3CF2-08B3-4D15-882C-6B0BBFCA97B5}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5380A27B-2D7E-4002-B459-EBE5044FFD9F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9462631-6499-4C1A-8B40-8D442C38DA1C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D9CF7E2-B40D-410E-9074-10945FA93BCC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADE2C9DF-61C1-47B8-981E-A6BA85493504}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 22/07/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -1243,7 +1243,7 @@
     <t>130012843</t>
   </si>
   <si>
-    <t>UP BRASIL ADMINISTRACAO E SERVICOS LTDA.</t>
+    <t>UP BRASIL ADMINISTRACAO SERVICOS E INSTITUICAO DE PAGAMENTO LTDA</t>
   </si>
   <si>
     <t>02.959.392/0001-46</t>
@@ -56831,13 +56831,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DAFC3CF2-08B3-4D15-882C-6B0BBFCA97B5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93AFCA08-C5DF-4833-9297-2982A7DF6FD5}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9462631-6499-4C1A-8B40-8D442C38DA1C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{887386E8-1ED2-4B8B-8BEC-B2A916144E34}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADE2C9DF-61C1-47B8-981E-A6BA85493504}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9B1C188-6609-4A17-8760-0F8E441FEA8F}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 24/07/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -56831,13 +56831,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{93AFCA08-C5DF-4833-9297-2982A7DF6FD5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{88F22AEB-069C-4BEC-876C-B5ADF03051C4}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{887386E8-1ED2-4B8B-8BEC-B2A916144E34}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA4A1B73-24F3-4841-A4EF-842105C25A22}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9B1C188-6609-4A17-8760-0F8E441FEA8F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8B87560-5951-4897-B6E6-7EF9FC49024F}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 30/07/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -57059,13 +57059,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2278808F-D869-4933-8126-83893342E84E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73619CDA-8ED7-4E92-862D-929432DECEC4}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{777524A6-FFE4-4FF8-951F-2909FB4CE0F7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FE7F299-DF40-4E73-85F9-A8D61A91F2C5}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81A72BFF-ABE9-4ACF-B4A4-CA608B06B809}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA173F75-F8DD-4A7F-A821-338D71F5C5DB}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 31/07/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -57059,13 +57059,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73619CDA-8ED7-4E92-862D-929432DECEC4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B0159399-BCBA-40E8-B5C6-58DD04828540}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FE7F299-DF40-4E73-85F9-A8D61A91F2C5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15A67E25-F5F2-48F8-B5D7-39BAA83CEE8B}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA173F75-F8DD-4A7F-A821-338D71F5C5DB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97E01656-C2C4-4239-B4BB-E96991531D3C}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 21/08/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -59260,13 +59260,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF867B11-4F96-4539-881D-67645918DFA4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7A3608A6-8BFF-46E0-939D-3C72A68A9EA8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{532B9E83-08A7-4643-92D5-55106836DD19}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D26E7635-884B-41DB-B6AA-2B2FCFA304A2}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D50C6D48-B877-4913-BDEA-6E12B0964BE9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78586F2F-CAD8-47B0-8169-1E746678C5C6}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 27/08/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -43017,7 +43017,7 @@
         <v>5927</v>
       </c>
       <c r="V363" s="6">
-        <v>-693596</v>
+        <v>46259</v>
       </c>
       <c r="W363" s="4" t="s">
         <v>405</v>
@@ -44877,7 +44877,7 @@
         <v>5925</v>
       </c>
       <c r="V379" s="6">
-        <v>-693596</v>
+        <v>46259</v>
       </c>
       <c r="W379" s="4" t="s">
         <v>405</v>
@@ -44994,7 +44994,7 @@
         <v>5926</v>
       </c>
       <c r="V380" s="6">
-        <v>-693596</v>
+        <v>46259</v>
       </c>
       <c r="W380" s="4" t="s">
         <v>405</v>
@@ -45111,7 +45111,7 @@
         <v>5928</v>
       </c>
       <c r="V381" s="6">
-        <v>-693596</v>
+        <v>46259</v>
       </c>
       <c r="W381" s="4" t="s">
         <v>405</v>
@@ -59734,13 +59734,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1597378E-AA14-4637-BE04-0510EB2BA2F3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9BE5552B-2D47-4CC8-863D-19EE599C98BA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BED33E4A-98B0-48AA-8A19-B502682CABEA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E772B3E-46AB-45AD-807D-16116706FD9D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D15BEBD7-9675-4AB1-A7F6-6CD4E122A0F1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC7374DE-161A-4C22-AEDB-48D1F95128E8}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 31/08/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -59731,13 +59731,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F2130AA-B74F-4053-B9D6-93869E752ED0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F659F295-9DED-4A97-AACB-4477E289E3B3}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90A4D96F-4178-49BA-B360-3B02F70E1AB3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17CC1868-1E44-45FA-B831-C7F14F65A577}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55961EB1-A2A4-4024-B5AC-9FAEEB4B75FD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26BC60AD-018C-4AED-8B9B-274DEEDEC387}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 02/09/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -59731,13 +59731,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{10FBA239-18AD-4BE4-9AC7-67B8F15D62E4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42983305-BB0B-47F1-B3BB-F7ACBB763960}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3BD43C81-069B-4908-A127-8563580924AD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{965AAF34-2C11-41F9-9474-775EBCC2E4B3}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFDFCBDB-F0E7-4C64-9092-40A1C64ED922}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98F8973B-02B9-40BC-A804-FB17E09179B8}"/>
 </file>
</xml_diff>

<commit_message>
Atualizar restos.xlsx - 08/09/2026
</commit_message>
<xml_diff>
--- a/restos.xlsx
+++ b/restos.xlsx
@@ -59731,13 +59731,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42983305-BB0B-47F1-B3BB-F7ACBB763960}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEB9BBA4-2CE1-42C1-9974-D53B79C72EAE}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{965AAF34-2C11-41F9-9474-775EBCC2E4B3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2123FC4-845C-471F-9607-E8CC8BA56AFE}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98F8973B-02B9-40BC-A804-FB17E09179B8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32BD3B49-99FC-4F08-B6FE-395879FCAFA3}"/>
 </file>
</xml_diff>